<commit_message>
mise a jour docs
</commit_message>
<xml_diff>
--- a/docs/Planification.-P_OO_320-MartinIvliev-jnltrav_heures.xlsx
+++ b/docs/Planification.-P_OO_320-MartinIvliev-jnltrav_heures.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30621"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduvaud-my.sharepoint.com/personal/pm00buq_eduvaud_ch/Documents/Modules actifs/P_POO 320/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="418" documentId="8_{C5A1DFEF-2C38-4239-8B7B-364697EA1FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DF645F37-E0D2-47C5-9489-6CBFF10979AD}"/>
+  <xr:revisionPtr revIDLastSave="495" documentId="8_{C5A1DFEF-2C38-4239-8B7B-364697EA1FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{952A55E3-AD5F-4395-9623-348B9AE258E3}"/>
   <bookViews>
     <workbookView xWindow="32235" yWindow="3975" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="121">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -114,6 +114,9 @@
     <t>Analyse du projet</t>
   </si>
   <si>
+    <t>La presentation par le professeur / analyse</t>
+  </si>
+  <si>
     <t>2026-oo-parking-cdc.pdf</t>
   </si>
   <si>
@@ -141,43 +144,136 @@
     <t>Implementation de la planification</t>
   </si>
   <si>
+    <t>Analyse</t>
+  </si>
+  <si>
     <t>Implementation du rapport</t>
   </si>
   <si>
+    <t>Details sur le code</t>
+  </si>
+  <si>
     <t>Implementation du journal de travail</t>
   </si>
   <si>
     <t>Creation de la class voiture</t>
   </si>
   <si>
-    <t>Creation du tablo</t>
+    <t>Creation de la class voiture avec plaque.</t>
+  </si>
+  <si>
+    <t>Creation du tableau</t>
+  </si>
+  <si>
+    <t>Creation tableau pour afficher la place de la voiture.</t>
   </si>
   <si>
     <t>Creation du menu</t>
   </si>
   <si>
+    <t>Creation du menu pour afficher les options possibles.</t>
+  </si>
+  <si>
     <t>Option sortie</t>
   </si>
   <si>
-    <t xml:space="preserve"> ajoute de l option de sortie en verifiant que la plaque soit bien dans le tablo des vehicules</t>
-  </si>
-  <si>
-    <t>sortie du vehicule</t>
-  </si>
-  <si>
-    <t>Option affichage de tablo</t>
-  </si>
-  <si>
-    <t>affichage en pourcentage et vehicules presents</t>
-  </si>
-  <si>
-    <t>tablo qui affiche tout seul automatiquement tout les vehicules garee</t>
-  </si>
-  <si>
-    <t>statistiques</t>
-  </si>
-  <si>
-    <t>recherche</t>
+    <t>Ajoute de l option de sortie en verifiant que la plaque soit bien dans le tablo des vehicules.</t>
+  </si>
+  <si>
+    <t>Sortie du vehicule en le suppriment du tableau.</t>
+  </si>
+  <si>
+    <t>Option affichage de Tableau</t>
+  </si>
+  <si>
+    <t>Affichage en pourcentage et vehicules presents.</t>
+  </si>
+  <si>
+    <t>Tableau qui affiche tout seul automatiquement tout les vehicules garee.</t>
+  </si>
+  <si>
+    <t>Class statistiques</t>
+  </si>
+  <si>
+    <t>Class statistique qui grace aux calcules affiche les statistiques du parking.</t>
+  </si>
+  <si>
+    <t>Class recherche</t>
+  </si>
+  <si>
+    <t>Class recherche qui parcours tout les plaque des vehicules / places pour montrer le ticket du vehicule en question.</t>
+  </si>
+  <si>
+    <t>Corriection des bugs</t>
+  </si>
+  <si>
+    <t>Suppresion des boucles inutiles.</t>
+  </si>
+  <si>
+    <t>Amelioration du code</t>
+  </si>
+  <si>
+    <t>Correction des bugs.</t>
+  </si>
+  <si>
+    <t>Amelioration generalle</t>
+  </si>
+  <si>
+    <t>Ajout de la classe parking et random</t>
+  </si>
+  <si>
+    <t>Ajout de la calsse parking pour afficher les places et random pour créer des nombres aleatoires.</t>
+  </si>
+  <si>
+    <t>Correction pour les normes de nommage de l'etml</t>
+  </si>
+  <si>
+    <t>remise des variables et methodes en anglais / majuscules pour les variables statiques / _ (tiré du bas) pour les variables privées</t>
+  </si>
+  <si>
+    <t>Ajout des commentaires explicatifs</t>
+  </si>
+  <si>
+    <t>ajout des commentaire pour expliquer comment fonctionne chaque methode / objet</t>
+  </si>
+  <si>
+    <t>Ajout de l encapsulation</t>
+  </si>
+  <si>
+    <t>ajout de get et set</t>
+  </si>
+  <si>
+    <t>Test unitaire pour verifier la plaque d'immatriculation</t>
+  </si>
+  <si>
+    <t>tests</t>
+  </si>
+  <si>
+    <t>Sortie du vehicule correction</t>
+  </si>
+  <si>
+    <t>Sortie du vehicule corrigé et avec verification si l'utilisateur mets un chiffre(place) ou la plaque d'immatriculation(demandé a l'ia isnullorwhitespace).</t>
+  </si>
+  <si>
+    <t>Terminer Historique</t>
+  </si>
+  <si>
+    <t>Methode historique</t>
+  </si>
+  <si>
+    <t>Ajout de controle de plaque correcte</t>
+  </si>
+  <si>
+    <t>Controle de plaque complet</t>
+  </si>
+  <si>
+    <t>Ajustement methode sortie</t>
+  </si>
+  <si>
+    <t>correction de la methode qui prenait pas en compte la plaque</t>
+  </si>
+  <si>
+    <t>Ajustement code</t>
   </si>
   <si>
     <t>Total en heures</t>
@@ -658,51 +754,51 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1035,10 +1131,10 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="30"/>
+      <c r="C1" s="39"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
@@ -1050,10 +1146,10 @@
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="30"/>
+      <c r="C2" s="39"/>
       <c r="D2" s="22" t="s">
         <v>6</v>
       </c>
@@ -1065,10 +1161,10 @@
       <c r="A3" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="30"/>
+      <c r="C3" s="39"/>
       <c r="D3" s="22" t="s">
         <v>10</v>
       </c>
@@ -1080,12 +1176,12 @@
       <c r="A4" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="33"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1">
       <c r="A5" s="2" t="s">
@@ -1108,35 +1204,37 @@
       <c r="A6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="40">
+      <c r="B6" s="30">
         <v>46262</v>
       </c>
       <c r="C6" s="5">
         <v>45</v>
       </c>
-      <c r="D6" s="6"/>
+      <c r="D6" s="6" t="s">
+        <v>20</v>
+      </c>
       <c r="E6" s="25" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="35"/>
+        <v>22</v>
+      </c>
+      <c r="B7" s="31"/>
       <c r="C7" s="8">
         <v>10</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="23" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="35"/>
+        <v>24</v>
+      </c>
+      <c r="B8" s="31"/>
       <c r="C8" s="8">
         <v>20</v>
       </c>
@@ -1145,22 +1243,22 @@
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1">
       <c r="A9" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="35"/>
+        <v>25</v>
+      </c>
+      <c r="B9" s="31"/>
       <c r="C9" s="8">
         <v>30</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="25" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1">
       <c r="A10" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="36"/>
+        <v>27</v>
+      </c>
+      <c r="B10" s="32"/>
       <c r="C10" s="10">
         <v>30</v>
       </c>
@@ -1169,42 +1267,46 @@
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A11" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="37"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B11" s="33"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="35"/>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="40">
+        <v>29</v>
+      </c>
+      <c r="B12" s="30">
         <v>46269</v>
       </c>
       <c r="C12" s="5">
         <v>45</v>
       </c>
-      <c r="D12" s="6"/>
+      <c r="D12" s="6" t="s">
+        <v>30</v>
+      </c>
       <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1">
       <c r="A13" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="35"/>
+        <v>31</v>
+      </c>
+      <c r="B13" s="31"/>
       <c r="C13" s="8">
         <v>45</v>
       </c>
-      <c r="D13" s="9"/>
+      <c r="D13" s="9" t="s">
+        <v>32</v>
+      </c>
       <c r="E13" s="8"/>
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="35"/>
+        <v>33</v>
+      </c>
+      <c r="B14" s="31"/>
       <c r="C14" s="8">
         <v>45</v>
       </c>
@@ -1213,9 +1315,9 @@
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1">
       <c r="A15" s="7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="35"/>
+        <v>29</v>
+      </c>
+      <c r="B15" s="31"/>
       <c r="C15" s="8">
         <v>45</v>
       </c>
@@ -1224,58 +1326,64 @@
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A16" s="10"/>
-      <c r="B16" s="36"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="10"/>
       <c r="D16" s="11"/>
       <c r="E16" s="10"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1">
       <c r="A17" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="37"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B17" s="33"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="35"/>
     </row>
     <row r="18" spans="1:5" ht="18" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="B18" s="40">
+        <v>34</v>
+      </c>
+      <c r="B18" s="30">
         <v>46276</v>
       </c>
       <c r="C18" s="5">
         <v>45</v>
       </c>
-      <c r="D18" s="6"/>
+      <c r="D18" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="E18" s="5"/>
     </row>
     <row r="19" spans="1:5" ht="18" customHeight="1">
       <c r="A19" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B19" s="35"/>
+        <v>36</v>
+      </c>
+      <c r="B19" s="31"/>
       <c r="C19" s="8">
         <v>45</v>
       </c>
-      <c r="D19" s="9"/>
+      <c r="D19" s="9" t="s">
+        <v>37</v>
+      </c>
       <c r="E19" s="8"/>
     </row>
     <row r="20" spans="1:5" ht="18" customHeight="1">
       <c r="A20" s="7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B20" s="35"/>
+        <v>38</v>
+      </c>
+      <c r="B20" s="31"/>
       <c r="C20" s="8">
         <v>45</v>
       </c>
-      <c r="D20" s="9"/>
+      <c r="D20" s="9" t="s">
+        <v>39</v>
+      </c>
       <c r="E20" s="8"/>
     </row>
     <row r="21" spans="1:5" ht="18" customHeight="1">
       <c r="A21" s="7"/>
-      <c r="B21" s="35"/>
+      <c r="B21" s="31"/>
       <c r="C21" s="8">
         <v>45</v>
       </c>
@@ -1284,167 +1392,181 @@
     </row>
     <row r="22" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A22" s="10"/>
-      <c r="B22" s="36"/>
+      <c r="B22" s="32"/>
       <c r="C22" s="10"/>
       <c r="D22" s="11"/>
       <c r="E22" s="10"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1">
       <c r="A23" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B23" s="37"/>
-      <c r="C23" s="38"/>
-      <c r="D23" s="38"/>
-      <c r="E23" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B23" s="33"/>
+      <c r="C23" s="34"/>
+      <c r="D23" s="34"/>
+      <c r="E23" s="35"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1">
       <c r="A24" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B24" s="40">
+        <v>40</v>
+      </c>
+      <c r="B24" s="30">
         <v>46283</v>
       </c>
       <c r="C24" s="5">
         <v>45</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E24" s="5"/>
     </row>
     <row r="25" spans="1:5" ht="18" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B25" s="35"/>
+        <v>40</v>
+      </c>
+      <c r="B25" s="31"/>
       <c r="C25" s="8">
         <v>45</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E25" s="8"/>
     </row>
     <row r="26" spans="1:5" ht="18" customHeight="1">
       <c r="A26" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B26" s="35"/>
+        <v>43</v>
+      </c>
+      <c r="B26" s="31"/>
       <c r="C26" s="8">
         <v>45</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E26" s="8"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1">
       <c r="A27" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B27" s="35"/>
+        <v>43</v>
+      </c>
+      <c r="B27" s="31"/>
       <c r="C27" s="8">
         <v>45</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E27" s="8"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1">
       <c r="A28" s="10"/>
-      <c r="B28" s="36"/>
+      <c r="B28" s="32"/>
       <c r="C28" s="10"/>
       <c r="D28" s="11"/>
       <c r="E28" s="10"/>
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A29" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B29" s="37"/>
-      <c r="C29" s="38"/>
-      <c r="D29" s="38"/>
-      <c r="E29" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B29" s="33"/>
+      <c r="C29" s="34"/>
+      <c r="D29" s="34"/>
+      <c r="E29" s="35"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1">
       <c r="A30" s="13" t="s">
-        <v>40</v>
-      </c>
-      <c r="B30" s="40">
+        <v>46</v>
+      </c>
+      <c r="B30" s="30">
         <v>46290</v>
       </c>
       <c r="C30" s="13">
         <v>45</v>
       </c>
-      <c r="D30" s="14"/>
+      <c r="D30" s="14" t="s">
+        <v>47</v>
+      </c>
       <c r="E30" s="13"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1">
       <c r="A31" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="B31" s="35"/>
+        <v>48</v>
+      </c>
+      <c r="B31" s="31"/>
       <c r="C31" s="8">
         <v>45</v>
       </c>
-      <c r="D31" s="9"/>
+      <c r="D31" s="9" t="s">
+        <v>49</v>
+      </c>
       <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" ht="18" customHeight="1">
       <c r="A32" s="8"/>
-      <c r="B32" s="35"/>
+      <c r="B32" s="31"/>
       <c r="C32" s="8"/>
       <c r="D32" s="9"/>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="18" customHeight="1">
       <c r="A33" s="8"/>
-      <c r="B33" s="35"/>
+      <c r="B33" s="31"/>
       <c r="C33" s="8"/>
       <c r="D33" s="9"/>
       <c r="E33" s="8"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A34" s="8"/>
-      <c r="B34" s="36"/>
+      <c r="B34" s="32"/>
       <c r="C34" s="8"/>
       <c r="D34" s="9"/>
       <c r="E34" s="8"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1">
       <c r="A35" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B35" s="37"/>
-      <c r="C35" s="38"/>
-      <c r="D35" s="38"/>
-      <c r="E35" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B35" s="33"/>
+      <c r="C35" s="34"/>
+      <c r="D35" s="34"/>
+      <c r="E35" s="35"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1">
-      <c r="A36" s="8"/>
-      <c r="B36" s="40">
+      <c r="A36" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="B36" s="30">
         <v>46297</v>
       </c>
       <c r="C36" s="5">
         <v>45</v>
       </c>
-      <c r="D36" s="6"/>
+      <c r="D36" s="6" t="s">
+        <v>51</v>
+      </c>
       <c r="E36" s="5"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1">
-      <c r="A37" s="8"/>
-      <c r="B37" s="35"/>
+      <c r="A37" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="B37" s="31"/>
       <c r="C37" s="8">
         <v>45</v>
       </c>
-      <c r="D37" s="9"/>
+      <c r="D37" s="9" t="s">
+        <v>53</v>
+      </c>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1">
-      <c r="A38" s="8"/>
-      <c r="B38" s="35"/>
+      <c r="A38" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B38" s="31"/>
       <c r="C38" s="8">
         <v>45</v>
       </c>
@@ -1452,227 +1574,281 @@
       <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" ht="18" customHeight="1">
-      <c r="A39" s="8"/>
-      <c r="B39" s="35"/>
+      <c r="A39" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B39" s="31"/>
       <c r="C39" s="8">
         <v>45</v>
       </c>
-      <c r="D39" s="9"/>
+      <c r="D39" s="9" t="s">
+        <v>56</v>
+      </c>
       <c r="E39" s="8"/>
     </row>
     <row r="40" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A40" s="8"/>
-      <c r="B40" s="36"/>
-      <c r="C40" s="10">
-        <v>45</v>
-      </c>
+      <c r="B40" s="32"/>
+      <c r="C40" s="10"/>
       <c r="D40" s="11"/>
       <c r="E40" s="10"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A41" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B41" s="37"/>
-      <c r="C41" s="38"/>
-      <c r="D41" s="38"/>
-      <c r="E41" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B41" s="33"/>
+      <c r="C41" s="34"/>
+      <c r="D41" s="34"/>
+      <c r="E41" s="35"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1">
-      <c r="A42" s="4"/>
-      <c r="B42" s="40">
-        <v>45721</v>
-      </c>
-      <c r="C42" s="5"/>
-      <c r="D42" s="6"/>
+      <c r="A42" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="B42" s="30">
+        <v>46299</v>
+      </c>
+      <c r="C42" s="5">
+        <v>45</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>58</v>
+      </c>
       <c r="E42" s="5"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1">
-      <c r="A43" s="7"/>
-      <c r="B43" s="35"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="9"/>
+      <c r="A43" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="B43" s="31"/>
+      <c r="C43" s="8">
+        <v>20</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>60</v>
+      </c>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1">
-      <c r="A44" s="7"/>
-      <c r="B44" s="35"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="9"/>
+      <c r="A44" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B44" s="31"/>
+      <c r="C44" s="8">
+        <v>20</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>62</v>
+      </c>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1">
       <c r="A45" s="7"/>
-      <c r="B45" s="35"/>
+      <c r="B45" s="31"/>
       <c r="C45" s="8"/>
       <c r="D45" s="9"/>
       <c r="E45" s="8"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A46" s="10"/>
-      <c r="B46" s="36"/>
+      <c r="B46" s="32"/>
       <c r="C46" s="10"/>
       <c r="D46" s="11"/>
       <c r="E46" s="10"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A47" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B47" s="37"/>
-      <c r="C47" s="38"/>
-      <c r="D47" s="38"/>
-      <c r="E47" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B47" s="33"/>
+      <c r="C47" s="34"/>
+      <c r="D47" s="34"/>
+      <c r="E47" s="35"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1">
-      <c r="A48" s="4"/>
-      <c r="B48" s="40">
-        <v>46093</v>
-      </c>
-      <c r="C48" s="5"/>
-      <c r="D48" s="6"/>
+      <c r="A48" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="B48" s="30">
+        <v>46300</v>
+      </c>
+      <c r="C48" s="5">
+        <v>90</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>64</v>
+      </c>
       <c r="E48" s="5"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1">
-      <c r="A49" s="7"/>
-      <c r="B49" s="35"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="9"/>
+      <c r="A49" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="B49" s="31"/>
+      <c r="C49" s="8">
+        <v>45</v>
+      </c>
+      <c r="D49" s="9" t="s">
+        <v>66</v>
+      </c>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1">
       <c r="A50" s="7"/>
-      <c r="B50" s="35"/>
+      <c r="B50" s="31"/>
       <c r="C50" s="8"/>
       <c r="D50" s="9"/>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1">
       <c r="A51" s="7"/>
-      <c r="B51" s="35"/>
+      <c r="B51" s="31"/>
       <c r="C51" s="8"/>
       <c r="D51" s="9"/>
       <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A52" s="10"/>
-      <c r="B52" s="36"/>
+      <c r="B52" s="32"/>
       <c r="C52" s="10"/>
       <c r="D52" s="11"/>
       <c r="E52" s="10"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A53" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B53" s="37"/>
-      <c r="C53" s="38"/>
-      <c r="D53" s="38"/>
-      <c r="E53" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B53" s="33"/>
+      <c r="C53" s="34"/>
+      <c r="D53" s="34"/>
+      <c r="E53" s="35"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1">
-      <c r="A54" s="4"/>
-      <c r="B54" s="34"/>
-      <c r="C54" s="5"/>
-      <c r="D54" s="6"/>
+      <c r="A54" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B54" s="30">
+        <v>46325</v>
+      </c>
+      <c r="C54" s="5">
+        <v>45</v>
+      </c>
+      <c r="D54" s="6" t="s">
+        <v>68</v>
+      </c>
       <c r="E54" s="5"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1">
-      <c r="A55" s="7"/>
-      <c r="B55" s="35"/>
-      <c r="C55" s="8"/>
-      <c r="D55" s="9"/>
+      <c r="A55" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="B55" s="31"/>
+      <c r="C55" s="8">
+        <v>45</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>70</v>
+      </c>
       <c r="E55" s="8"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1">
-      <c r="A56" s="7"/>
-      <c r="B56" s="35"/>
-      <c r="C56" s="8"/>
-      <c r="D56" s="9"/>
+      <c r="A56" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B56" s="31"/>
+      <c r="C56" s="8">
+        <v>45</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>72</v>
+      </c>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1">
-      <c r="A57" s="7"/>
-      <c r="B57" s="35"/>
+      <c r="A57" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="B57" s="31"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A58" s="10"/>
-      <c r="B58" s="36"/>
+      <c r="B58" s="32"/>
       <c r="C58" s="10"/>
       <c r="D58" s="11"/>
       <c r="E58" s="10"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A59" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B59" s="37"/>
-      <c r="C59" s="38"/>
-      <c r="D59" s="38"/>
-      <c r="E59" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B59" s="33"/>
+      <c r="C59" s="34"/>
+      <c r="D59" s="34"/>
+      <c r="E59" s="35"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1">
       <c r="A60" s="13"/>
-      <c r="B60" s="34"/>
+      <c r="B60" s="38"/>
       <c r="C60" s="13"/>
       <c r="D60" s="14"/>
       <c r="E60" s="13"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1">
       <c r="A61" s="8"/>
-      <c r="B61" s="35"/>
+      <c r="B61" s="31"/>
       <c r="C61" s="8"/>
       <c r="D61" s="9"/>
       <c r="E61" s="8"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1">
       <c r="A62" s="8"/>
-      <c r="B62" s="35"/>
+      <c r="B62" s="31"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1">
       <c r="A63" s="8"/>
-      <c r="B63" s="35"/>
+      <c r="B63" s="31"/>
       <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A64" s="8"/>
-      <c r="B64" s="36"/>
+      <c r="B64" s="32"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A65" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B65" s="37"/>
-      <c r="C65" s="38"/>
-      <c r="D65" s="38"/>
-      <c r="E65" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B65" s="33"/>
+      <c r="C65" s="34"/>
+      <c r="D65" s="34"/>
+      <c r="E65" s="35"/>
     </row>
     <row r="66" spans="1:5" ht="21" customHeight="1" thickBot="1">
-      <c r="A66" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="B66" s="42"/>
+      <c r="A66" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="B66" s="37"/>
       <c r="C66" s="15">
         <f>MROUND(SUM(C6:C65) /60,0.2)</f>
-        <v>16.600000000000001</v>
+        <v>21.6</v>
       </c>
       <c r="D66" s="16"/>
       <c r="E66" s="17"/>
     </row>
     <row r="68" spans="1:5">
       <c r="A68" s="18" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
     </row>
     <row r="69" spans="1:5">
@@ -1680,15 +1856,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="B36:B40"/>
-    <mergeCell ref="B65:E65"/>
-    <mergeCell ref="A66:B66"/>
-    <mergeCell ref="B42:B46"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B48:B52"/>
-    <mergeCell ref="B53:E53"/>
-    <mergeCell ref="B54:B58"/>
-    <mergeCell ref="B59:E59"/>
     <mergeCell ref="B1:C1"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="B3:C3"/>
@@ -1705,6 +1872,15 @@
     <mergeCell ref="B29:E29"/>
     <mergeCell ref="B30:B34"/>
     <mergeCell ref="B35:E35"/>
+    <mergeCell ref="B36:B40"/>
+    <mergeCell ref="B65:E65"/>
+    <mergeCell ref="A66:B66"/>
+    <mergeCell ref="B42:B46"/>
+    <mergeCell ref="B47:E47"/>
+    <mergeCell ref="B48:B52"/>
+    <mergeCell ref="B53:E53"/>
+    <mergeCell ref="B54:B58"/>
+    <mergeCell ref="B59:E59"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="C54:C58 C48:C52 C36:C40 C42:C46 C18:C22 B6 C12:C16 C24:C28 C30:C34 C60:C64 C6:C10" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1751,25 +1927,25 @@
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="30" t="s">
+      <c r="B1" s="39" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="30"/>
+      <c r="C1" s="39"/>
       <c r="D1" s="22" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="20" t="s">
-        <v>44</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="21" customHeight="1" thickBot="1">
       <c r="A2" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="30" t="s">
+      <c r="B2" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="30"/>
+      <c r="C2" s="39"/>
       <c r="D2" s="22" t="s">
         <v>6</v>
       </c>
@@ -1781,10 +1957,10 @@
       <c r="A3" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="39" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="30"/>
+      <c r="C3" s="39"/>
       <c r="D3" s="22" t="s">
         <v>10</v>
       </c>
@@ -1796,12 +1972,12 @@
       <c r="A4" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="40" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="32"/>
-      <c r="D4" s="32"/>
-      <c r="E4" s="33"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="42"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1">
       <c r="A5" s="2" t="s">
@@ -1824,7 +2000,7 @@
       <c r="A6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="40">
+      <c r="B6" s="30">
         <v>46262</v>
       </c>
       <c r="C6" s="5">
@@ -1832,40 +2008,40 @@
       </c>
       <c r="D6" s="6"/>
       <c r="E6" s="24" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1">
       <c r="A7" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="35"/>
+        <v>22</v>
+      </c>
+      <c r="B7" s="31"/>
       <c r="C7" s="8">
         <v>5</v>
       </c>
       <c r="D7" s="9"/>
       <c r="E7" s="23" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1">
       <c r="A8" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="35"/>
+        <v>24</v>
+      </c>
+      <c r="B8" s="31"/>
       <c r="C8" s="8">
         <v>30</v>
       </c>
       <c r="D8" s="9"/>
       <c r="E8" s="27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1">
       <c r="A9" s="7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" s="35"/>
+        <v>25</v>
+      </c>
+      <c r="B9" s="31"/>
       <c r="C9" s="8">
         <v>30</v>
       </c>
@@ -1874,9 +2050,9 @@
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A10" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="36"/>
+        <v>27</v>
+      </c>
+      <c r="B10" s="32"/>
       <c r="C10" s="10">
         <v>30</v>
       </c>
@@ -1885,18 +2061,18 @@
     </row>
     <row r="11" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A11" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="37"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B11" s="33"/>
+      <c r="C11" s="34"/>
+      <c r="D11" s="34"/>
+      <c r="E11" s="35"/>
     </row>
     <row r="12" spans="1:5" ht="18" customHeight="1">
       <c r="A12" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="40">
+        <v>29</v>
+      </c>
+      <c r="B12" s="30">
         <v>46269</v>
       </c>
       <c r="C12" s="5">
@@ -1907,9 +2083,9 @@
     </row>
     <row r="13" spans="1:5" ht="18" customHeight="1">
       <c r="A13" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="35"/>
+        <v>31</v>
+      </c>
+      <c r="B13" s="31"/>
       <c r="C13" s="8">
         <v>45</v>
       </c>
@@ -1918,9 +2094,9 @@
     </row>
     <row r="14" spans="1:5" ht="18" customHeight="1">
       <c r="A14" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="35"/>
+        <v>33</v>
+      </c>
+      <c r="B14" s="31"/>
       <c r="C14" s="8">
         <v>45</v>
       </c>
@@ -1929,32 +2105,32 @@
     </row>
     <row r="15" spans="1:5" ht="18" customHeight="1">
       <c r="A15" s="7"/>
-      <c r="B15" s="35"/>
+      <c r="B15" s="31"/>
       <c r="C15" s="8"/>
       <c r="D15" s="9"/>
       <c r="E15" s="8"/>
     </row>
     <row r="16" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A16" s="10"/>
-      <c r="B16" s="36"/>
+      <c r="B16" s="32"/>
       <c r="C16" s="10"/>
       <c r="D16" s="11"/>
       <c r="E16" s="10"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1">
       <c r="A17" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="37"/>
-      <c r="C17" s="38"/>
-      <c r="D17" s="38"/>
-      <c r="E17" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B17" s="33"/>
+      <c r="C17" s="34"/>
+      <c r="D17" s="34"/>
+      <c r="E17" s="35"/>
     </row>
     <row r="18" spans="1:5" ht="45" customHeight="1">
       <c r="A18" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B18" s="40">
+        <v>78</v>
+      </c>
+      <c r="B18" s="30">
         <v>46276</v>
       </c>
       <c r="C18" s="5">
@@ -1965,59 +2141,59 @@
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1">
       <c r="A19" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B19" s="35"/>
+        <v>79</v>
+      </c>
+      <c r="B19" s="31"/>
       <c r="C19" s="8">
         <v>20</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>48</v>
+        <v>80</v>
       </c>
       <c r="E19" s="8"/>
     </row>
     <row r="20" spans="1:5" ht="27.75" customHeight="1">
       <c r="A20" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B20" s="35"/>
+        <v>81</v>
+      </c>
+      <c r="B20" s="31"/>
       <c r="C20" s="8">
         <v>45</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>50</v>
+        <v>82</v>
       </c>
       <c r="E20" s="8"/>
     </row>
     <row r="21" spans="1:5" ht="50.25" customHeight="1">
       <c r="A21" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="B21" s="35"/>
+        <v>83</v>
+      </c>
+      <c r="B21" s="31"/>
       <c r="C21" s="8">
         <v>45</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>52</v>
+        <v>84</v>
       </c>
       <c r="E21" s="8"/>
     </row>
     <row r="22" spans="1:5" ht="44.25" customHeight="1">
       <c r="A22" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="B22" s="36"/>
+        <v>85</v>
+      </c>
+      <c r="B22" s="32"/>
       <c r="C22" s="10">
         <v>45</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>54</v>
+        <v>86</v>
       </c>
       <c r="E22" s="10"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>55</v>
+        <v>87</v>
       </c>
       <c r="B23" s="26">
         <v>46276</v>
@@ -2026,372 +2202,372 @@
         <v>15</v>
       </c>
       <c r="D23" s="28" t="s">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="E23" s="28"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1">
       <c r="A24" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B24" s="37"/>
-      <c r="C24" s="38"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B24" s="33"/>
+      <c r="C24" s="34"/>
+      <c r="D24" s="34"/>
+      <c r="E24" s="35"/>
     </row>
     <row r="25" spans="1:5" ht="38.25" customHeight="1">
       <c r="A25" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="B25" s="40">
+        <v>89</v>
+      </c>
+      <c r="B25" s="30">
         <v>46283</v>
       </c>
       <c r="C25" s="5">
         <v>45</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="E25" s="5"/>
     </row>
     <row r="26" spans="1:5" ht="27.75" customHeight="1">
       <c r="A26" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B26" s="35"/>
+        <v>91</v>
+      </c>
+      <c r="B26" s="31"/>
       <c r="C26" s="8">
         <v>45</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>60</v>
+        <v>92</v>
       </c>
       <c r="E26" s="8"/>
     </row>
     <row r="27" spans="1:5" ht="29.25" customHeight="1">
       <c r="A27" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="B27" s="35"/>
+        <v>93</v>
+      </c>
+      <c r="B27" s="31"/>
       <c r="C27" s="8">
         <v>45</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>62</v>
+        <v>94</v>
       </c>
       <c r="E27" s="8"/>
     </row>
     <row r="28" spans="1:5" ht="25.5" customHeight="1">
       <c r="A28" s="4" t="s">
-        <v>63</v>
-      </c>
-      <c r="B28" s="35"/>
+        <v>95</v>
+      </c>
+      <c r="B28" s="31"/>
       <c r="C28" s="8">
         <v>30</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="E28" s="8"/>
     </row>
     <row r="29" spans="1:5" ht="18" customHeight="1">
       <c r="A29" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="B29" s="36"/>
+        <v>87</v>
+      </c>
+      <c r="B29" s="32"/>
       <c r="C29" s="10">
         <v>15</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="E29" s="10"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1">
       <c r="A30" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B30" s="37"/>
-      <c r="C30" s="38"/>
-      <c r="D30" s="38"/>
-      <c r="E30" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B30" s="33"/>
+      <c r="C30" s="34"/>
+      <c r="D30" s="34"/>
+      <c r="E30" s="35"/>
     </row>
     <row r="31" spans="1:5" ht="45" customHeight="1">
       <c r="A31" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="B31" s="40">
+        <v>97</v>
+      </c>
+      <c r="B31" s="30">
         <v>46290</v>
       </c>
       <c r="C31" s="13">
         <v>45</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>66</v>
+        <v>98</v>
       </c>
       <c r="E31" s="13"/>
     </row>
     <row r="32" spans="1:5" ht="34.5" customHeight="1">
       <c r="A32" s="13" t="s">
-        <v>67</v>
-      </c>
-      <c r="B32" s="35"/>
+        <v>99</v>
+      </c>
+      <c r="B32" s="31"/>
       <c r="C32" s="8">
         <v>60</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>68</v>
+        <v>100</v>
       </c>
       <c r="E32" s="8"/>
     </row>
     <row r="33" spans="1:5" ht="39.75" customHeight="1">
       <c r="A33" s="13" t="s">
-        <v>69</v>
-      </c>
-      <c r="B33" s="35"/>
+        <v>101</v>
+      </c>
+      <c r="B33" s="31"/>
       <c r="C33" s="8">
         <v>60</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>70</v>
+        <v>102</v>
       </c>
       <c r="E33" s="8"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1">
       <c r="A34" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="B34" s="35"/>
+        <v>87</v>
+      </c>
+      <c r="B34" s="31"/>
       <c r="C34" s="8">
         <v>15</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="E34" s="8"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A35" s="8"/>
-      <c r="B35" s="36"/>
+      <c r="B35" s="32"/>
       <c r="C35" s="8"/>
       <c r="D35" s="9"/>
       <c r="E35" s="8"/>
     </row>
     <row r="36" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A36" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B36" s="37"/>
-      <c r="C36" s="38"/>
-      <c r="D36" s="38"/>
-      <c r="E36" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B36" s="33"/>
+      <c r="C36" s="34"/>
+      <c r="D36" s="34"/>
+      <c r="E36" s="35"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1">
       <c r="A37" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B37" s="40">
+        <v>103</v>
+      </c>
+      <c r="B37" s="30">
         <v>46297</v>
       </c>
       <c r="C37" s="5">
         <v>30</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>72</v>
+        <v>104</v>
       </c>
       <c r="E37" s="5"/>
     </row>
     <row r="38" spans="1:5" ht="32.25" customHeight="1">
       <c r="A38" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="B38" s="35"/>
+        <v>105</v>
+      </c>
+      <c r="B38" s="31"/>
       <c r="C38" s="8">
         <v>45</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="E38" s="8"/>
     </row>
     <row r="39" spans="1:5" ht="26.25" customHeight="1">
       <c r="A39" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="B39" s="35"/>
+        <v>107</v>
+      </c>
+      <c r="B39" s="31"/>
       <c r="C39" s="8">
         <v>45</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="E39" s="8"/>
     </row>
     <row r="40" spans="1:5" ht="40.5" customHeight="1">
       <c r="A40" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B40" s="35"/>
+        <v>109</v>
+      </c>
+      <c r="B40" s="31"/>
       <c r="C40" s="8">
         <v>45</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>78</v>
+        <v>110</v>
       </c>
       <c r="E40" s="8"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1">
       <c r="A41" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="B41" s="36"/>
+        <v>87</v>
+      </c>
+      <c r="B41" s="32"/>
       <c r="C41" s="10">
         <v>15</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="E41" s="10"/>
     </row>
     <row r="42" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A42" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B42" s="37"/>
-      <c r="C42" s="38"/>
-      <c r="D42" s="38"/>
-      <c r="E42" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B42" s="33"/>
+      <c r="C42" s="34"/>
+      <c r="D42" s="34"/>
+      <c r="E42" s="35"/>
     </row>
     <row r="43" spans="1:5" ht="37.5" customHeight="1">
       <c r="A43" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="B43" s="40">
+        <v>111</v>
+      </c>
+      <c r="B43" s="30">
         <v>46304</v>
       </c>
       <c r="C43" s="5">
         <v>75</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>80</v>
+        <v>112</v>
       </c>
       <c r="E43" s="5"/>
     </row>
     <row r="44" spans="1:5" ht="59.25" customHeight="1">
       <c r="A44" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="B44" s="35"/>
+        <v>113</v>
+      </c>
+      <c r="B44" s="31"/>
       <c r="C44" s="8">
         <v>75</v>
       </c>
       <c r="D44" s="6" t="s">
-        <v>82</v>
+        <v>114</v>
       </c>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1">
       <c r="A45" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B45" s="35"/>
+        <v>87</v>
+      </c>
+      <c r="B45" s="31"/>
       <c r="C45" s="8">
         <v>15</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>56</v>
+        <v>88</v>
       </c>
       <c r="E45" s="8"/>
     </row>
     <row r="46" spans="1:5" ht="18" customHeight="1">
       <c r="A46" s="7"/>
-      <c r="B46" s="35"/>
+      <c r="B46" s="31"/>
       <c r="C46" s="8"/>
       <c r="D46" s="9"/>
       <c r="E46" s="8"/>
     </row>
     <row r="47" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A47" s="10"/>
-      <c r="B47" s="36"/>
+      <c r="B47" s="32"/>
       <c r="C47" s="10"/>
       <c r="D47" s="11"/>
       <c r="E47" s="10"/>
     </row>
     <row r="48" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A48" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B48" s="37"/>
-      <c r="C48" s="38"/>
-      <c r="D48" s="38"/>
-      <c r="E48" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B48" s="33"/>
+      <c r="C48" s="34"/>
+      <c r="D48" s="34"/>
+      <c r="E48" s="35"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1">
       <c r="A49" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B49" s="40">
+        <v>115</v>
+      </c>
+      <c r="B49" s="30">
         <v>46311</v>
       </c>
       <c r="C49" s="5">
         <v>45</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>84</v>
+        <v>116</v>
       </c>
       <c r="E49" s="5"/>
     </row>
     <row r="50" spans="1:5" ht="30.75" customHeight="1">
       <c r="A50" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="B50" s="35"/>
+        <v>117</v>
+      </c>
+      <c r="B50" s="31"/>
       <c r="C50" s="8">
         <v>45</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>86</v>
+        <v>118</v>
       </c>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="42.75" customHeight="1">
       <c r="A51" s="29" t="s">
-        <v>87</v>
-      </c>
-      <c r="B51" s="35"/>
+        <v>119</v>
+      </c>
+      <c r="B51" s="31"/>
       <c r="C51" s="8">
         <v>45</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>88</v>
+        <v>120</v>
       </c>
       <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1">
       <c r="A52" s="7"/>
-      <c r="B52" s="35"/>
+      <c r="B52" s="31"/>
       <c r="C52" s="8"/>
       <c r="D52" s="9"/>
       <c r="E52" s="8"/>
     </row>
     <row r="53" spans="1:5" ht="18" customHeight="1" thickBot="1">
       <c r="A53" s="10"/>
-      <c r="B53" s="36"/>
+      <c r="B53" s="32"/>
       <c r="C53" s="10"/>
       <c r="D53" s="11"/>
       <c r="E53" s="10"/>
     </row>
     <row r="54" spans="1:5" ht="18" customHeight="1">
       <c r="A54" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B54" s="37"/>
-      <c r="C54" s="38"/>
-      <c r="D54" s="38"/>
-      <c r="E54" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B54" s="33"/>
+      <c r="C54" s="34"/>
+      <c r="D54" s="34"/>
+      <c r="E54" s="35"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1">
       <c r="A55" s="4"/>
-      <c r="B55" s="40">
+      <c r="B55" s="30">
         <v>46318</v>
       </c>
       <c r="C55" s="5"/>
@@ -2400,44 +2576,44 @@
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1">
       <c r="A56" s="7"/>
-      <c r="B56" s="35"/>
+      <c r="B56" s="31"/>
       <c r="C56" s="8"/>
       <c r="D56" s="9"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1">
       <c r="A57" s="7"/>
-      <c r="B57" s="35"/>
+      <c r="B57" s="31"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1">
       <c r="A58" s="7"/>
-      <c r="B58" s="35"/>
+      <c r="B58" s="31"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1">
       <c r="A59" s="10"/>
-      <c r="B59" s="36"/>
+      <c r="B59" s="32"/>
       <c r="C59" s="10"/>
       <c r="D59" s="11"/>
       <c r="E59" s="10"/>
     </row>
     <row r="60" spans="1:5" ht="18" customHeight="1">
       <c r="A60" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B60" s="37"/>
-      <c r="C60" s="38"/>
-      <c r="D60" s="38"/>
-      <c r="E60" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B60" s="33"/>
+      <c r="C60" s="34"/>
+      <c r="D60" s="34"/>
+      <c r="E60" s="35"/>
     </row>
     <row r="61" spans="1:5" ht="18" customHeight="1">
       <c r="A61" s="13"/>
-      <c r="B61" s="40">
+      <c r="B61" s="30">
         <v>46325</v>
       </c>
       <c r="C61" s="13"/>
@@ -2446,46 +2622,46 @@
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1">
       <c r="A62" s="8"/>
-      <c r="B62" s="35"/>
+      <c r="B62" s="31"/>
       <c r="C62" s="8"/>
       <c r="D62" s="9"/>
       <c r="E62" s="8"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1">
       <c r="A63" s="8"/>
-      <c r="B63" s="35"/>
+      <c r="B63" s="31"/>
       <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1">
       <c r="A64" s="8"/>
-      <c r="B64" s="35"/>
+      <c r="B64" s="31"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1">
       <c r="A65" s="8"/>
-      <c r="B65" s="36"/>
+      <c r="B65" s="32"/>
       <c r="C65" s="8"/>
       <c r="D65" s="9"/>
       <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1">
       <c r="A66" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="B66" s="37"/>
-      <c r="C66" s="38"/>
-      <c r="D66" s="38"/>
-      <c r="E66" s="39"/>
+        <v>28</v>
+      </c>
+      <c r="B66" s="33"/>
+      <c r="C66" s="34"/>
+      <c r="D66" s="34"/>
+      <c r="E66" s="35"/>
     </row>
     <row r="67" spans="1:5" ht="21" customHeight="1" thickBot="1">
-      <c r="A67" s="41" t="s">
-        <v>42</v>
-      </c>
-      <c r="B67" s="42"/>
+      <c r="A67" s="36" t="s">
+        <v>74</v>
+      </c>
+      <c r="B67" s="37"/>
       <c r="C67" s="15">
         <f>MROUND(SUM(C6:C66) /60,0.2)</f>
         <v>21.6</v>
@@ -2495,7 +2671,7 @@
     </row>
     <row r="69" spans="1:5">
       <c r="A69" s="18" t="s">
-        <v>43</v>
+        <v>75</v>
       </c>
     </row>
     <row r="70" spans="1:5">
@@ -2503,13 +2679,12 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A67:B67"/>
-    <mergeCell ref="B49:B53"/>
-    <mergeCell ref="B54:E54"/>
-    <mergeCell ref="B55:B59"/>
-    <mergeCell ref="B60:E60"/>
-    <mergeCell ref="B61:B65"/>
-    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B11:E11"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="B6:B10"/>
     <mergeCell ref="B48:E48"/>
     <mergeCell ref="B12:B16"/>
     <mergeCell ref="B17:E17"/>
@@ -2522,12 +2697,13 @@
     <mergeCell ref="B37:B41"/>
     <mergeCell ref="B42:E42"/>
     <mergeCell ref="B43:B47"/>
-    <mergeCell ref="B11:E11"/>
-    <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B6:B10"/>
+    <mergeCell ref="A67:B67"/>
+    <mergeCell ref="B49:B53"/>
+    <mergeCell ref="B54:E54"/>
+    <mergeCell ref="B55:B59"/>
+    <mergeCell ref="B60:E60"/>
+    <mergeCell ref="B61:B65"/>
+    <mergeCell ref="B66:E66"/>
   </mergeCells>
   <dataValidations count="2">
     <dataValidation type="date" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B12:B16 B55:B59 B25:B29 B31:B35 B37:B41 B43:B47 B49:B53 B18:B23 B61:B65" xr:uid="{EE54CF5D-239E-4F78-8D4F-7AFBFF2A539C}">
@@ -2554,6 +2730,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -2715,15 +2900,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
@@ -2731,11 +2907,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>